<commit_message>
Excel import fixes: allow large sheets (172 KB request was refused), free-text review status, unknown quantity accepted and flagged, time-of-day no longer shifts dates, order refs for existing orders
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/subcontractor-template.xlsx
+++ b/frontend/subcontractor-template.xlsx
@@ -231,7 +231,7 @@
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Required quantity (pcs), more than 0. Required.</t>
+        <t>Required quantity (pcs). Leave blank while it is not known: the order is flagged until you enter it.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
@@ -291,7 +291,7 @@
     </comment>
     <comment ref="V1" authorId="0" shapeId="0">
       <text>
-        <t>Rich review status.</t>
+        <t>Review status with Rich. Suggested: SUBMITTED, IN REVIEW, CHANGES REQUESTED, APPROVED. Other wording is kept as written.</t>
       </text>
     </comment>
     <comment ref="W1" authorId="0" shapeId="0">
@@ -636,7 +636,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
@@ -694,7 +694,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
@@ -16990,7 +16990,7 @@
       <formula1>DATE(2000,1,1)</formula1>
       <formula2>DATE(2100,12,31)</formula2>
     </dataValidation>
-    <dataValidation sqref="V2:V501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Choose from the list" error="Pick one of: SUBMITTED, IN REVIEW, CHANGES REQUESTED, APPROVED" type="list">
+    <dataValidation sqref="V2:V501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the suggested list" error="Other wording is allowed. Keep it as it is?" type="list" errorStyle="warning">
       <formula1>"SUBMITTED,IN REVIEW,CHANGES REQUESTED,APPROVED"</formula1>
     </dataValidation>
     <dataValidation sqref="W2:W501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date" error="Enter a date, for example 2026-11-30." type="date" operator="between">
@@ -17303,19 +17303,19 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>Qty *</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>Order</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>Required quantity (pcs), more than 0. Required.</t>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Required quantity (pcs). Leave blank while it is not known: the order is flagged until you enter it.</t>
         </is>
       </c>
     </row>
@@ -17604,7 +17604,7 @@
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Rich review status. Allowed: SUBMITTED, IN REVIEW, CHANGES REQUESTED, APPROVED.</t>
+          <t>Review status with Rich. Suggested: SUBMITTED, IN REVIEW, CHANGES REQUESTED, APPROVED. Other wording is kept as written.</t>
         </is>
       </c>
     </row>

</xml_diff>